<commit_message>
slight update to Version Record
</commit_message>
<xml_diff>
--- a/Version_Record.xlsx
+++ b/Version_Record.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\km154756\KagglePlaygroundS05E05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{217212DA-B604-48BF-BEC7-CA88124CBBA2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDC52413-C4CD-4A21-90D2-59F0B44C1E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{192F5873-E18C-4183-90A3-7D5AEEBF95A6}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="108" uniqueCount="40">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="41">
   <si>
     <t>Features</t>
   </si>
@@ -156,10 +156,16 @@
     <t>see Version 4</t>
   </si>
   <si>
-    <t>test predictions stored in V8_submissions.csv</t>
-  </si>
-  <si>
     <t>Hill Starting Equal</t>
+  </si>
+  <si>
+    <t>CatBoost(0.38077869) 
+XGB(0.38153654)
+LGBM(0.23768477)</t>
+  </si>
+  <si>
+    <t>CatBoost(0.51251431) 
+XGB(0.48748569)</t>
   </si>
 </sst>
 </file>
@@ -270,8 +276,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D7588A39-CF0D-4F28-887C-4CD75967C9DB}" name="Table1" displayName="Table1" ref="A1:N9" totalsRowShown="0" dataDxfId="14">
-  <autoFilter ref="A1:N9" xr:uid="{D7588A39-CF0D-4F28-887C-4CD75967C9DB}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D7588A39-CF0D-4F28-887C-4CD75967C9DB}" name="Table1" displayName="Table1" ref="A1:N8" totalsRowShown="0" dataDxfId="14">
+  <autoFilter ref="A1:N8" xr:uid="{D7588A39-CF0D-4F28-887C-4CD75967C9DB}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{90FE3CD3-65F1-4940-84BE-3084D27B4E8C}" name="Version" dataDxfId="13"/>
     <tableColumn id="2" xr3:uid="{1E95F86C-8266-47AE-A6C1-8D2CAABE8413}" name="Features" dataDxfId="12"/>
@@ -609,20 +615,20 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FD47C56-92A0-402D-93B8-FA89A7088413}">
-  <dimension ref="A1:N9"/>
+  <dimension ref="A1:N8"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
     <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="44.5703125" customWidth="1"/>
-    <col min="6" max="6" width="28.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="42.42578125" customWidth="1"/>
+    <col min="6" max="6" width="26.42578125" style="3" customWidth="1"/>
     <col min="7" max="7" width="20.42578125" customWidth="1"/>
     <col min="8" max="8" width="19.140625" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18.42578125" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="19.42578125" customWidth="1"/>
-    <col min="11" max="11" width="20.42578125" customWidth="1"/>
+    <col min="10" max="10" width="13.85546875" customWidth="1"/>
+    <col min="11" max="11" width="13.42578125" customWidth="1"/>
     <col min="12" max="12" width="18.85546875" customWidth="1"/>
     <col min="13" max="13" width="14.5703125" customWidth="1"/>
     <col min="14" max="14" width="20" bestFit="1" customWidth="1"/>
@@ -873,7 +879,7 @@
         <v>21</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="I6" s="2" t="s">
         <v>30</v>
@@ -894,7 +900,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="7" spans="1:14" ht="45" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:14" ht="60" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
@@ -917,20 +923,22 @@
         <v>31</v>
       </c>
       <c r="H7" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="I7" s="1"/>
       <c r="J7" s="1" t="s">
         <v>11</v>
       </c>
       <c r="K7" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="L7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M7" s="1" t="s">
-        <v>11</v>
+      <c r="L7" s="1">
+        <v>5.9193000000000003E-2</v>
+      </c>
+      <c r="M7" s="1">
+        <v>5.679E-2</v>
       </c>
       <c r="N7" s="2" t="s">
         <v>32</v>
@@ -947,7 +955,7 @@
         <v>10</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="E8" s="2" t="s">
         <v>37</v>
@@ -961,63 +969,23 @@
       <c r="H8" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="I8" s="1"/>
+      <c r="I8" s="2" t="s">
+        <v>40</v>
+      </c>
       <c r="J8" s="1" t="s">
         <v>11</v>
       </c>
       <c r="K8" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="L8" s="1" t="s">
-        <v>11</v>
+      <c r="L8" s="1">
+        <v>5.9277000000000003E-2</v>
       </c>
       <c r="M8" s="1" t="s">
         <v>11</v>
       </c>
       <c r="N8" s="2" t="s">
         <v>36</v>
-      </c>
-    </row>
-    <row r="9" spans="1:14" ht="45" x14ac:dyDescent="0.25">
-      <c r="A9" s="1">
-        <v>8</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="I9" s="1"/>
-      <c r="J9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="K9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="L9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="M9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="N9" s="2" t="s">
-        <v>38</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
changes to new.ipynb as well as new notebooks for hyperparameter optimization
</commit_message>
<xml_diff>
--- a/Version_Record.xlsx
+++ b/Version_Record.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\km154756\KagglePlaygroundS05E05\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDC52413-C4CD-4A21-90D2-59F0B44C1E37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BD9D96C3-A58B-45D1-9A98-F8CB2EF4F866}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{192F5873-E18C-4183-90A3-7D5AEEBF95A6}"/>
+    <workbookView xWindow="45972" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{192F5873-E18C-4183-90A3-7D5AEEBF95A6}"/>
   </bookViews>
   <sheets>
     <sheet name="Versions" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="95" uniqueCount="41">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="53">
   <si>
     <t>Features</t>
   </si>
@@ -51,9 +51,6 @@
   </si>
   <si>
     <t>Cross-Validation</t>
-  </si>
-  <si>
-    <t>Ridge/Hill</t>
   </si>
   <si>
     <t>Outlier Ensemble</t>
@@ -156,9 +153,6 @@
     <t>see Version 4</t>
   </si>
   <si>
-    <t>Hill Starting Equal</t>
-  </si>
-  <si>
     <t>CatBoost(0.38077869) 
 XGB(0.38153654)
 LGBM(0.23768477)</t>
@@ -166,6 +160,50 @@
   <si>
     <t>CatBoost(0.51251431) 
 XGB(0.48748569)</t>
+  </si>
+  <si>
+    <t>XGB + CatBoost +LGBM + RFR</t>
+  </si>
+  <si>
+    <t>see Version 4 + RFR(n_estimators=500, max_depth=10, min_samples_split=10, min_samples_leaf=4, max_features='sqrt', random_state=42, n_jobs=-1)</t>
+  </si>
+  <si>
+    <t>Ignore</t>
+  </si>
+  <si>
+    <t>XGB + CatBoost + LGBM</t>
+  </si>
+  <si>
+    <t>All KFOLD(100)</t>
+  </si>
+  <si>
+    <t>test predictions stored in V8_submissions.csv</t>
+  </si>
+  <si>
+    <t>CatBoost(0.38851004)
+XGB(0.37918227)
+LGBM(0.2323077)</t>
+  </si>
+  <si>
+    <t>Verion6 + KaggleExample2 (Can Ozen)</t>
+  </si>
+  <si>
+    <t>See Version 6 + KaggleExample2</t>
+  </si>
+  <si>
+    <t>Both KFOLD(50)</t>
+  </si>
+  <si>
+    <t>None for overall (Hill for Version 6)</t>
+  </si>
+  <si>
+    <t>Version 6(0.45) + KaggleExample2(o.55)</t>
+  </si>
+  <si>
+    <t>test predictions stored in K2_V6submission.csv</t>
+  </si>
+  <si>
+    <t>Weighting Algorithm</t>
   </si>
 </sst>
 </file>
@@ -227,28 +265,28 @@
       <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <alignment horizontal="left" vertical="top" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
@@ -276,23 +314,23 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D7588A39-CF0D-4F28-887C-4CD75967C9DB}" name="Table1" displayName="Table1" ref="A1:N8" totalsRowShown="0" dataDxfId="14">
-  <autoFilter ref="A1:N8" xr:uid="{D7588A39-CF0D-4F28-887C-4CD75967C9DB}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{D7588A39-CF0D-4F28-887C-4CD75967C9DB}" name="Table1" displayName="Table1" ref="A1:N11" totalsRowShown="0" dataDxfId="14">
+  <autoFilter ref="A1:N11" xr:uid="{D7588A39-CF0D-4F28-887C-4CD75967C9DB}"/>
   <tableColumns count="14">
     <tableColumn id="1" xr3:uid="{90FE3CD3-65F1-4940-84BE-3084D27B4E8C}" name="Version" dataDxfId="13"/>
     <tableColumn id="2" xr3:uid="{1E95F86C-8266-47AE-A6C1-8D2CAABE8413}" name="Features" dataDxfId="12"/>
     <tableColumn id="3" xr3:uid="{5B18D934-C434-422F-BE53-CABF3195544C}" name="Target" dataDxfId="11"/>
     <tableColumn id="4" xr3:uid="{F3C59205-8B79-4D48-8B79-C5947E2509E6}" name="Models" dataDxfId="10"/>
-    <tableColumn id="5" xr3:uid="{B60D89E3-53F9-4813-B104-A78488DB4CCB}" name="HyperParameters" dataDxfId="2"/>
-    <tableColumn id="14" xr3:uid="{6287C065-9554-47E5-B14E-51A963001669}" name="HyperParameter Reasoning" dataDxfId="0"/>
-    <tableColumn id="6" xr3:uid="{C35B677C-F27C-46EC-A4E7-0910111E1E21}" name="Cross-Validation" dataDxfId="1"/>
-    <tableColumn id="7" xr3:uid="{253E3BD1-491C-4330-A613-ABEA215F5C56}" name="Ridge/Hill" dataDxfId="9"/>
-    <tableColumn id="13" xr3:uid="{A836A89C-33F7-4EF3-AB86-12D4603A473B}" name="Model Weighting" dataDxfId="8"/>
-    <tableColumn id="8" xr3:uid="{48923D1F-116A-424E-B48D-330122F0FBA0}" name="Outlier Ensemble" dataDxfId="7"/>
-    <tableColumn id="9" xr3:uid="{63DF656D-346E-49BD-B148-A370B9418951}" name="Training Bins" dataDxfId="6"/>
-    <tableColumn id="10" xr3:uid="{4EFB7799-F19A-4A7D-868A-CFAD836F2BA3}" name="Train Performance" dataDxfId="5"/>
-    <tableColumn id="12" xr3:uid="{B8C39B51-7DB8-4BB2-86C4-BC50DFCB3B5F}" name="Test Performance" dataDxfId="4"/>
-    <tableColumn id="11" xr3:uid="{9701B1D9-FFB3-4303-91BF-2ACE7A13BAA4}" name="Comments" dataDxfId="3"/>
+    <tableColumn id="5" xr3:uid="{B60D89E3-53F9-4813-B104-A78488DB4CCB}" name="HyperParameters" dataDxfId="9"/>
+    <tableColumn id="14" xr3:uid="{6287C065-9554-47E5-B14E-51A963001669}" name="HyperParameter Reasoning" dataDxfId="8"/>
+    <tableColumn id="6" xr3:uid="{C35B677C-F27C-46EC-A4E7-0910111E1E21}" name="Cross-Validation" dataDxfId="7"/>
+    <tableColumn id="7" xr3:uid="{253E3BD1-491C-4330-A613-ABEA215F5C56}" name="Weighting Algorithm" dataDxfId="6"/>
+    <tableColumn id="13" xr3:uid="{A836A89C-33F7-4EF3-AB86-12D4603A473B}" name="Model Weighting" dataDxfId="5"/>
+    <tableColumn id="8" xr3:uid="{48923D1F-116A-424E-B48D-330122F0FBA0}" name="Outlier Ensemble" dataDxfId="4"/>
+    <tableColumn id="9" xr3:uid="{63DF656D-346E-49BD-B148-A370B9418951}" name="Training Bins" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{4EFB7799-F19A-4A7D-868A-CFAD836F2BA3}" name="Train Performance" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{B8C39B51-7DB8-4BB2-86C4-BC50DFCB3B5F}" name="Test Performance" dataDxfId="1"/>
+    <tableColumn id="11" xr3:uid="{9701B1D9-FFB3-4303-91BF-2ACE7A13BAA4}" name="Comments" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -615,13 +653,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4FD47C56-92A0-402D-93B8-FA89A7088413}">
-  <dimension ref="A1:N8"/>
+  <dimension ref="A1:N11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="11" customWidth="1"/>
     <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="25.28515625" customWidth="1"/>
     <col min="5" max="5" width="42.42578125" customWidth="1"/>
     <col min="6" max="6" width="26.42578125" style="3" customWidth="1"/>
     <col min="7" max="7" width="20.42578125" customWidth="1"/>
@@ -629,7 +667,7 @@
     <col min="9" max="9" width="18.42578125" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.85546875" customWidth="1"/>
     <col min="11" max="11" width="13.42578125" customWidth="1"/>
-    <col min="12" max="12" width="18.85546875" customWidth="1"/>
+    <col min="12" max="12" width="19.7109375" customWidth="1"/>
     <col min="13" max="13" width="14.5703125" customWidth="1"/>
     <col min="14" max="14" width="20" bestFit="1" customWidth="1"/>
     <col min="15" max="15" width="24.28515625" customWidth="1"/>
@@ -638,7 +676,7 @@
   <sheetData>
     <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B1" t="s">
         <v>0</v>
@@ -653,31 +691,31 @@
         <v>3</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G1" t="s">
         <v>4</v>
       </c>
       <c r="H1" t="s">
+        <v>52</v>
+      </c>
+      <c r="I1" t="s">
+        <v>23</v>
+      </c>
+      <c r="J1" t="s">
         <v>5</v>
       </c>
-      <c r="I1" t="s">
-        <v>24</v>
-      </c>
-      <c r="J1" t="s">
+      <c r="K1" t="s">
         <v>6</v>
       </c>
-      <c r="K1" t="s">
-        <v>7</v>
-      </c>
       <c r="L1" t="s">
+        <v>13</v>
+      </c>
+      <c r="M1" t="s">
         <v>14</v>
       </c>
-      <c r="M1" t="s">
-        <v>15</v>
-      </c>
       <c r="N1" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="2" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -685,43 +723,43 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="D2" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F2" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L2" s="1">
         <v>6.0371000000000001E-2</v>
       </c>
       <c r="M2" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="3" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -729,43 +767,43 @@
         <v>2</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F3" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L3" s="1">
         <v>6.0044E-2</v>
       </c>
       <c r="M3" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
     </row>
     <row r="4" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -773,43 +811,43 @@
         <v>3</v>
       </c>
       <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C4" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="D4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="F4" s="2" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L4" s="1">
         <v>6.0005999999999997E-2</v>
       </c>
       <c r="M4" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="5" spans="1:14" ht="165" customHeight="1" x14ac:dyDescent="0.25">
@@ -817,34 +855,34 @@
         <v>4</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C5" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="D5" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F5" s="2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L5" s="1">
         <v>5.9326999999999998E-2</v>
@@ -853,7 +891,7 @@
         <v>5.6910000000000002E-2</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
     </row>
     <row r="6" spans="1:14" ht="60" x14ac:dyDescent="0.25">
@@ -861,34 +899,34 @@
         <v>5</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="D6" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F6" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>38</v>
+        <v>28</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L6" s="1">
         <v>5.9322E-2</v>
@@ -897,7 +935,7 @@
         <v>5.6869999999999997E-2</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="7" spans="1:14" ht="60" x14ac:dyDescent="0.25">
@@ -905,34 +943,34 @@
         <v>6</v>
       </c>
       <c r="B7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C7" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="D7" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I7" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>37</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="H7" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="I7" s="2" t="s">
-        <v>39</v>
-      </c>
       <c r="J7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L7" s="1">
         <v>5.9193000000000003E-2</v>
@@ -941,7 +979,7 @@
         <v>5.679E-2</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="8" spans="1:14" ht="45" x14ac:dyDescent="0.25">
@@ -949,43 +987,173 @@
         <v>7</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C8" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="C8" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="D8" s="1" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="F8" s="2" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="L8" s="1">
         <v>5.9277000000000003E-2</v>
       </c>
       <c r="M8" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="9" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A9" s="1">
+        <v>8</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="J9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K9" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="M9" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="N9" s="2"/>
+    </row>
+    <row r="10" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A10" s="1">
+        <v>9</v>
+      </c>
+      <c r="B10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="I10" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="J10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K10" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L10" s="1">
+        <v>5.9182999999999999E-2</v>
+      </c>
+      <c r="M10" s="1">
+        <v>5.6809999999999999E-2</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="11" spans="1:14" ht="60" x14ac:dyDescent="0.25">
+      <c r="A11" s="1">
         <v>11</v>
       </c>
-      <c r="N8" s="2" t="s">
-        <v>36</v>
+      <c r="B11" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G11" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="I11" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="J11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="K11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="L11" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="M11" s="1">
+        <v>5.6730000000000003E-2</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>51</v>
       </c>
     </row>
   </sheetData>

</xml_diff>